<commit_message>
final_valid_merged file created, 휴일 보정
</commit_message>
<xml_diff>
--- a/data/total_latest.xlsx
+++ b/data/total_latest.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I869"/>
+  <dimension ref="A1:I876"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25064,10 +25064,10 @@
         <v>46142</v>
       </c>
       <c r="B850" t="n">
-        <v>21014</v>
+        <v>21013</v>
       </c>
       <c r="C850" t="n">
-        <v>8574</v>
+        <v>8573</v>
       </c>
       <c r="D850" t="n">
         <v>9804</v>
@@ -25082,7 +25082,7 @@
         <v>1486</v>
       </c>
       <c r="H850" t="n">
-        <v>18378</v>
+        <v>18377</v>
       </c>
       <c r="I850" t="n">
         <v>22</v>
@@ -25528,7 +25528,7 @@
         <v>46158</v>
       </c>
       <c r="B866" t="n">
-        <v>15617</v>
+        <v>15616</v>
       </c>
       <c r="C866" t="n">
         <v>7543</v>
@@ -25543,13 +25543,13 @@
         <v>0</v>
       </c>
       <c r="G866" t="n">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H866" t="n">
         <v>14497</v>
       </c>
       <c r="I866" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="867">
@@ -25586,25 +25586,25 @@
         <v>46160</v>
       </c>
       <c r="B868" t="n">
-        <v>23810</v>
+        <v>23728</v>
       </c>
       <c r="C868" t="n">
         <v>8213</v>
       </c>
       <c r="D868" t="n">
-        <v>7964</v>
+        <v>7963</v>
       </c>
       <c r="E868" t="n">
-        <v>1773</v>
+        <v>1703</v>
       </c>
       <c r="F868" t="n">
         <v>1114</v>
       </c>
       <c r="G868" t="n">
-        <v>4746</v>
+        <v>4735</v>
       </c>
       <c r="H868" t="n">
-        <v>16177</v>
+        <v>16176</v>
       </c>
       <c r="I868" t="n">
         <v>23</v>
@@ -25615,28 +25615,231 @@
         <v>46161</v>
       </c>
       <c r="B869" t="n">
-        <v>23189</v>
+        <v>23091</v>
       </c>
       <c r="C869" t="n">
         <v>8054</v>
       </c>
       <c r="D869" t="n">
-        <v>9311</v>
+        <v>9309</v>
       </c>
       <c r="E869" t="n">
-        <v>1127</v>
+        <v>1043</v>
       </c>
       <c r="F869" t="n">
         <v>542</v>
       </c>
       <c r="G869" t="n">
-        <v>4155</v>
+        <v>4143</v>
       </c>
       <c r="H869" t="n">
-        <v>17365</v>
+        <v>17363</v>
       </c>
       <c r="I869" t="n">
         <v>25</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B870" t="n">
+        <v>21985</v>
+      </c>
+      <c r="C870" t="n">
+        <v>8171</v>
+      </c>
+      <c r="D870" t="n">
+        <v>9268</v>
+      </c>
+      <c r="E870" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F870" t="n">
+        <v>463</v>
+      </c>
+      <c r="G870" t="n">
+        <v>3060</v>
+      </c>
+      <c r="H870" t="n">
+        <v>17439</v>
+      </c>
+      <c r="I870" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="1" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B871" t="n">
+        <v>23700</v>
+      </c>
+      <c r="C871" t="n">
+        <v>9139</v>
+      </c>
+      <c r="D871" t="n">
+        <v>10441</v>
+      </c>
+      <c r="E871" t="n">
+        <v>1003</v>
+      </c>
+      <c r="F871" t="n">
+        <v>293</v>
+      </c>
+      <c r="G871" t="n">
+        <v>2824</v>
+      </c>
+      <c r="H871" t="n">
+        <v>19580</v>
+      </c>
+      <c r="I871" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="1" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B872" t="n">
+        <v>23222</v>
+      </c>
+      <c r="C872" t="n">
+        <v>8983</v>
+      </c>
+      <c r="D872" t="n">
+        <v>10651</v>
+      </c>
+      <c r="E872" t="n">
+        <v>709</v>
+      </c>
+      <c r="F872" t="n">
+        <v>295</v>
+      </c>
+      <c r="G872" t="n">
+        <v>2584</v>
+      </c>
+      <c r="H872" t="n">
+        <v>19634</v>
+      </c>
+      <c r="I872" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="1" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B873" t="n">
+        <v>16511</v>
+      </c>
+      <c r="C873" t="n">
+        <v>7479</v>
+      </c>
+      <c r="D873" t="n">
+        <v>7896</v>
+      </c>
+      <c r="E873" t="n">
+        <v>224</v>
+      </c>
+      <c r="F873" t="n">
+        <v>2</v>
+      </c>
+      <c r="G873" t="n">
+        <v>910</v>
+      </c>
+      <c r="H873" t="n">
+        <v>15375</v>
+      </c>
+      <c r="I873" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="1" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B874" t="n">
+        <v>13110</v>
+      </c>
+      <c r="C874" t="n">
+        <v>6828</v>
+      </c>
+      <c r="D874" t="n">
+        <v>6155</v>
+      </c>
+      <c r="E874" t="n">
+        <v>0</v>
+      </c>
+      <c r="F874" t="n">
+        <v>1</v>
+      </c>
+      <c r="G874" t="n">
+        <v>126</v>
+      </c>
+      <c r="H874" t="n">
+        <v>12983</v>
+      </c>
+      <c r="I874" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="1" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B875" t="n">
+        <v>14816</v>
+      </c>
+      <c r="C875" t="n">
+        <v>7463</v>
+      </c>
+      <c r="D875" t="n">
+        <v>6955</v>
+      </c>
+      <c r="E875" t="n">
+        <v>270</v>
+      </c>
+      <c r="F875" t="n">
+        <v>1</v>
+      </c>
+      <c r="G875" t="n">
+        <v>127</v>
+      </c>
+      <c r="H875" t="n">
+        <v>14418</v>
+      </c>
+      <c r="I875" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="1" t="n">
+        <v>46168</v>
+      </c>
+      <c r="B876" t="n">
+        <v>23965</v>
+      </c>
+      <c r="C876" t="n">
+        <v>8115</v>
+      </c>
+      <c r="D876" t="n">
+        <v>7818</v>
+      </c>
+      <c r="E876" t="n">
+        <v>1556</v>
+      </c>
+      <c r="F876" t="n">
+        <v>1272</v>
+      </c>
+      <c r="G876" t="n">
+        <v>5204</v>
+      </c>
+      <c r="H876" t="n">
+        <v>15933</v>
+      </c>
+      <c r="I876" t="n">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>